<commit_message>
fix(aud/of): clean residual PS/AU initials from DM7 footer signature
Audit found 2 hardcoded auditor initials (PS=preparador, AU=revisor) in
the DM7 Retenciones cédula footer signature cells (B75, B76). These
were leftovers from the original Moracosta template. Now both cells are
None — the assembler will overwrite them via HEADER_WRITES when the user
fills "prepared_by_name" and "reviewed_by_name" in the form.

Verified empirically (SHA256 before/after 3 sequential jobs): the
baked-in template file is NEVER modified during job execution. The
assembler loads the file, mutates an in-memory openpyxl Workbook,
and writes the result to BytesIO. Disk template stays read-only.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/app/aud/obligaciones_fiscales/templates/dm_obligaciones_fiscales.xlsx
+++ b/backend/app/aud/obligaciones_fiscales/templates/dm_obligaciones_fiscales.xlsx
@@ -3946,11 +3946,7 @@
         </is>
       </c>
       <c r="D24" s="193" t="n"/>
-      <c r="E24" s="388" t="inlineStr">
-        <is>
-          <t>JAUS</t>
-        </is>
-      </c>
+      <c r="E24" s="388" t="n"/>
       <c r="F24" s="63" t="n"/>
       <c r="G24" s="145" t="n"/>
     </row>
@@ -4752,6 +4748,8 @@
       </c>
       <c r="G28" s="332" t="n"/>
     </row>
+    <row r="29"/>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="326" t="inlineStr">
         <is>
@@ -8980,6 +8978,7 @@
       <c r="D9" s="162" t="n"/>
       <c r="E9" s="196" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="207" t="n"/>
       <c r="B11" s="208" t="n"/>
@@ -10059,6 +10058,7 @@
       <c r="L41" s="79" t="n"/>
       <c r="M41" s="80" t="n"/>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="A43" s="8" t="n"/>
     </row>
@@ -10508,6 +10508,8 @@
       <c r="E41" s="217" t="n"/>
     </row>
     <row r="42" ht="13.5" customHeight="1" thickTop="1"/>
+    <row r="43"/>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="170" t="inlineStr">
         <is>
@@ -10970,6 +10972,7 @@
       </c>
     </row>
     <row r="96" hidden="1" ht="13.5" customHeight="1" thickTop="1"/>
+    <row r="97"/>
     <row r="98">
       <c r="A98" s="8" t="n"/>
     </row>
@@ -12099,6 +12102,7 @@
       <c r="L35" s="31" t="n"/>
       <c r="M35" s="31" t="n"/>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="539" t="inlineStr">
         <is>
@@ -15124,6 +15128,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43">
       <c r="B43" s="8" t="inlineStr">
         <is>
@@ -15213,6 +15218,7 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
     <row r="46">
       <c r="A46" s="463" t="inlineStr">
         <is>
@@ -15676,6 +15682,7 @@
         <v/>
       </c>
     </row>
+    <row r="57"/>
     <row r="58">
       <c r="C58" s="2" t="n"/>
     </row>
@@ -34516,6 +34523,7 @@
       <c r="D10" s="541" t="n"/>
       <c r="E10" s="541" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
@@ -34542,6 +34550,7 @@
       <c r="C14" s="275" t="n"/>
       <c r="D14" s="275" t="n"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
@@ -37110,17 +37119,16 @@
       <c r="A71" s="194" t="n"/>
       <c r="B71" s="8" t="n"/>
     </row>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="131" t="inlineStr">
         <is>
           <t>Elaborado por:</t>
         </is>
       </c>
-      <c r="B75" s="387" t="inlineStr">
-        <is>
-          <t>PS</t>
-        </is>
-      </c>
+      <c r="B75" s="387" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="131" t="inlineStr">
@@ -37128,11 +37136,7 @@
           <t>Revisado por:</t>
         </is>
       </c>
-      <c r="B76" s="387" t="inlineStr">
-        <is>
-          <t>AU</t>
-        </is>
-      </c>
+      <c r="B76" s="387" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="131" t="inlineStr">
@@ -40448,6 +40452,7 @@
         </is>
       </c>
     </row>
+    <row r="75"/>
     <row r="76" hidden="1">
       <c r="A76" s="233" t="inlineStr">
         <is>
@@ -40785,6 +40790,7 @@
       <c r="C84" s="217" t="n"/>
       <c r="H84" s="217" t="n"/>
     </row>
+    <row r="85"/>
     <row r="86">
       <c r="B86" s="32" t="inlineStr">
         <is>
@@ -41092,6 +41098,10 @@
         </is>
       </c>
     </row>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
     <row r="108">
       <c r="B108" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(aud/of): remove 12 embedded images leftover from Moracosta template
User found screenshot data showing "RENDIMIENTOS FINANCIEROS" with
Moracosta numbers (11M, 10M) embedded as IMAGE in DM5 Ventas — not in
cells. Previous audits only checked cell values, missing images entirely.

Audit found 12 embedded images total across all sheets:
- DM Programa, DM1, DM2, DM3, DM4: 1 image each
- DM5 Ventas: 2 images (the "more_ver" screenshot user saw)
- DM6, DM7, DM8, DM9, DM10: 1 image each

All removed. Template now has 0 embedded images. The firm logo
(audit_consulting OR partner_auditing) is inserted at runtime by
excel_assembler._insert_logo() — never baked into the template.

Template size: 277KB -> 117KB.
Demo verified: generated Excel has exactly 11 images (= logos of selected
firma_auditora, one per cédula sheet).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/app/aud/obligaciones_fiscales/templates/dm_obligaciones_fiscales.xlsx
+++ b/backend/app/aud/obligaciones_fiscales/templates/dm_obligaciones_fiscales.xlsx
@@ -2741,608 +2741,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>104775</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1483179</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="104775"/>
-          <a:ext cx="2245179" cy="704850"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>904874</colOff>
-      <row>1</row>
-      <rowOff>345281</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Imagen 9"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2028824" cy="792956"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1162050</colOff>
-      <row>1</row>
-      <rowOff>266700</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2390775" cy="685800"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>95250</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1721304</colOff>
-      <row>3</row>
-      <rowOff>28575</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="95250"/>
-          <a:ext cx="2245179" cy="781050"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>59531</colOff>
-      <row>0</row>
-      <rowOff>83344</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>690562</colOff>
-      <row>1</row>
-      <rowOff>229715</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Imagen 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="59531" y="83344"/>
-          <a:ext cx="2035969" cy="646434"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1290205</colOff>
-      <row>2</row>
-      <rowOff>294409</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2467841" cy="848591"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>666750</colOff>
-      <row>2</row>
-      <rowOff>333375</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Imagen 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2369344" cy="964406"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>1809750</colOff>
-      <row>2</row>
-      <rowOff>306915</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="2624667" cy="899582"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>517071</colOff>
-      <row>28</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>26</col>
-      <colOff>611333</colOff>
-      <row>37</row>
-      <rowOff>111381</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Imagen 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="19485428" y="5021036"/>
-          <a:ext cx="7904762" cy="1580952"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>1</col>
-      <colOff>710045</colOff>
-      <row>3</row>
-      <rowOff>17318</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="1827068" cy="961159"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>1</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>1466851</colOff>
-      <row>3</row>
-      <rowOff>9525</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="1" y="0"/>
-          <a:ext cx="1466850" cy="752475"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
-<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>0</col>
-      <colOff>3337428</colOff>
-      <row>13</row>
-      <rowOff>11906</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Imagen 2"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1" noChangeArrowheads="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <lum bright="70000" contrast="-70000"/>
-        </a:blip>
-        <a:srcRect xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr bwMode="auto">
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:off x="0" y="0"/>
-          <a:ext cx="3337428" cy="1059656"/>
-        </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:noFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
@@ -4220,7 +3618,6 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="60"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4748,8 +4145,6 @@
       </c>
       <c r="G28" s="332" t="n"/>
     </row>
-    <row r="29"/>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="326" t="inlineStr">
         <is>
@@ -6886,7 +6281,6 @@
     <mergeCell ref="B52:D52"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7079,7 +6473,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="64"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -7948,7 +7341,6 @@
     <brk id="8" min="0" max="1048575" man="1"/>
     <brk id="45" min="3" max="53" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8978,7 +8370,6 @@
       <c r="D9" s="162" t="n"/>
       <c r="E9" s="196" t="n"/>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="207" t="n"/>
       <c r="B11" s="208" t="n"/>
@@ -10058,7 +9449,6 @@
       <c r="L41" s="79" t="n"/>
       <c r="M41" s="80" t="n"/>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="8" t="n"/>
     </row>
@@ -10096,7 +9486,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="36"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -10508,8 +9897,6 @@
       <c r="E41" s="217" t="n"/>
     </row>
     <row r="42" ht="13.5" customHeight="1" thickTop="1"/>
-    <row r="43"/>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="170" t="inlineStr">
         <is>
@@ -10972,7 +10359,6 @@
       </c>
     </row>
     <row r="96" hidden="1" ht="13.5" customHeight="1" thickTop="1"/>
-    <row r="97"/>
     <row r="98">
       <c r="A98" s="8" t="n"/>
     </row>
@@ -11034,7 +10420,6 @@
   <colBreaks count="1" manualBreakCount="1">
     <brk id="4" min="0" max="1048575" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -12094,7 +11479,6 @@
       <c r="L35" s="31" t="n"/>
       <c r="M35" s="31" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="539" t="inlineStr">
         <is>
@@ -13638,7 +13022,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="36"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -15120,7 +14503,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="B43" s="8" t="inlineStr">
         <is>
@@ -15210,7 +14592,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="463" t="inlineStr">
         <is>
@@ -15674,7 +15055,6 @@
         <v/>
       </c>
     </row>
-    <row r="57"/>
     <row r="58">
       <c r="C58" s="2" t="n"/>
     </row>
@@ -15784,7 +15164,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" scale="25"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -33846,7 +33225,6 @@
   <colBreaks count="1" manualBreakCount="1">
     <brk id="32" min="0" max="1048575" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -34515,7 +33893,6 @@
       <c r="D10" s="541" t="n"/>
       <c r="E10" s="541" t="n"/>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
@@ -34542,7 +33919,6 @@
       <c r="C14" s="275" t="n"/>
       <c r="D14" s="275" t="n"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
@@ -37093,9 +36469,6 @@
       <c r="A71" s="194" t="n"/>
       <c r="B71" s="8" t="n"/>
     </row>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
     <row r="75">
       <c r="A75" s="131" t="inlineStr">
         <is>
@@ -37146,7 +36519,6 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" scale="32"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -40426,7 +39798,6 @@
         </is>
       </c>
     </row>
-    <row r="75"/>
     <row r="76" hidden="1">
       <c r="A76" s="233" t="inlineStr">
         <is>
@@ -40764,7 +40135,6 @@
       <c r="C84" s="217" t="n"/>
       <c r="H84" s="217" t="n"/>
     </row>
-    <row r="85"/>
     <row r="86">
       <c r="B86" s="32" t="inlineStr">
         <is>
@@ -41072,10 +40442,6 @@
         </is>
       </c>
     </row>
-    <row r="104"/>
-    <row r="105"/>
-    <row r="106"/>
-    <row r="107"/>
     <row r="108">
       <c r="B108" s="3" t="inlineStr">
         <is>
@@ -41155,6 +40521,5 @@
   <colBreaks count="1" manualBreakCount="1">
     <brk id="15" min="0" max="1048575" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>